<commit_message>
commit . entry and daily reports done
</commit_message>
<xml_diff>
--- a/canteen-react/public/report-template.xlsx
+++ b/canteen-react/public/report-template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCAC3959-B2FF-4881-81E1-125C35A30567}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07A950FA-58E5-4567-B08D-6D8F1162C88E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1273,7 +1273,10 @@
       <c r="B42" s="28"/>
       <c r="C42" s="28"/>
       <c r="D42" s="27"/>
-      <c r="E42" s="29"/>
+      <c r="E42" s="29">
+        <f>SUM(E36:E41)</f>
+        <v>0</v>
+      </c>
       <c r="G42" s="10" t="s">
         <v>34</v>
       </c>

</xml_diff>

<commit_message>
commit fix , maybe final
</commit_message>
<xml_diff>
--- a/canteen-react/public/report-template.xlsx
+++ b/canteen-react/public/report-template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07A950FA-58E5-4567-B08D-6D8F1162C88E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE7BB2A5-3099-4CEE-91C9-EA77D782829D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1277,15 +1277,21 @@
         <f>SUM(E36:E41)</f>
         <v>0</v>
       </c>
-      <c r="G42" s="10" t="s">
+      <c r="G42" s="25">
+        <v>7</v>
+      </c>
+      <c r="H42" s="4"/>
+      <c r="I42" s="24"/>
+      <c r="J42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="13.95" customHeight="1" thickBot="1">
+      <c r="G43" t="s">
         <v>34</v>
       </c>
-      <c r="H42" s="4"/>
-      <c r="I42" s="9">
-        <f>SUM(I36:I41)</f>
-        <v>0</v>
-      </c>
-      <c r="J42">
+      <c r="I43" s="9">
+        <f>SUM(I36:I42)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>